<commit_message>
feat(ui): link dashboard coverage gaps to workflow tabs
Add audit change-router skill, dashboard navigation, NCR a11y labels, and related test fixes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/release/xlsx-smoke.xlsx
+++ b/artifacts/release/xlsx-smoke.xlsx
@@ -272,7 +272,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve">王稽核</t>
+          <t xml:space="preserve">品保部經理</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -327,7 +327,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve">品保部經理</t>
+          <t xml:space="preserve">王稽核</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">

</xml_diff>

<commit_message>
feat(qms): add single-workspace migration and recovery
</commit_message>
<xml_diff>
--- a/artifacts/release/xlsx-smoke.xlsx
+++ b/artifacts/release/xlsx-smoke.xlsx
@@ -13,7 +13,6 @@
     <sheet name="觀察事項" sheetId="9" r:id="rId9"/>
     <sheet name="建議追蹤" sheetId="10" r:id="rId10"/>
     <sheet name="稽核前準備" sheetId="11" r:id="rId11"/>
-    <sheet name="外稽當日行程" sheetId="12" r:id="rId12"/>
   </sheets>
 </workbook>
 </file>
@@ -2048,25 +2047,10 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">九潤</t>
+          <t xml:space="preserve">完成</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">正隆興</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">合併</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">完成</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
         <is>
           <t xml:space="preserve">備註</t>
         </is>
@@ -2086,16 +2070,6 @@
           <t xml:space="preserve">品保/管理代表</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -2114,11 +2088,11 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">QR-28-03 稽核矯正報告（兩家各自備查）</t>
+          <t xml:space="preserve">QR-28-03 稽核矯正報告</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2129,11 +2103,11 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">QR-28-07 內外部稽核報告書（兩家各自備查）</t>
+          <t xml:space="preserve">QR-28-07 內外部稽核報告書</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2144,11 +2118,11 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">各部門年度目標訂定及統計分析完成/公告</t>
+          <t xml:space="preserve">各部門年度目標訂定及統計分析完成／公告</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2159,7 +2133,7 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -2174,7 +2148,7 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -2189,11 +2163,11 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">品質政策/品質目標之宣導及公告</t>
+          <t xml:space="preserve">品質政策／品質目標之宣導及公告</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2204,7 +2178,7 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -2219,7 +2193,7 @@
     </row>
     <row r="14">
       <c r="A14">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -2234,7 +2208,7 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -2249,11 +2223,11 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">機器設備保養記錄/相關指導書/標示等確認/模具區整理及標示確認</t>
+          <t xml:space="preserve">機器設備保養記錄／相關指導書／標示等確認／模具區整理及標示確認</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2264,11 +2238,11 @@
     </row>
     <row r="17">
       <c r="A17">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">各區域之標示區隔（進料/退貨/不合格品…等）</t>
+          <t xml:space="preserve">各區域之標示區隔（進料／退貨／不合格品…等）</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2279,7 +2253,7 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -2294,11 +2268,11 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">新產品送樣資料整理（MOT SOP/SIP/圖面/試製工單/首件/客戶核准樣品）</t>
+          <t xml:space="preserve">新產品送樣資料整理（MOT SOP／SIP／圖面／試製工單／首件／客戶核准樣品）</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2309,7 +2283,7 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -2324,7 +2298,7 @@
     </row>
     <row r="21">
       <c r="A21">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -2339,11 +2313,11 @@
     </row>
     <row r="22">
       <c r="A22">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">庫房/樣品之整理標示/記錄</t>
+          <t xml:space="preserve">庫房／樣品之整理標示／記錄</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2354,7 +2328,7 @@
     </row>
     <row r="23">
       <c r="A23">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2369,7 +2343,7 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2384,7 +2358,7 @@
     </row>
     <row r="25">
       <c r="A25">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2399,7 +2373,7 @@
     </row>
     <row r="26">
       <c r="A26">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2414,7 +2388,7 @@
     </row>
     <row r="27">
       <c r="A27">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2424,80 +2398,6 @@
       <c r="C27" t="inlineStr">
         <is>
           <t xml:space="preserve">品保</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外部稽核當日行程</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">年度：2026</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外稽日期：2026-09-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">日期</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">開始</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">結束</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">廠區</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">受稽單位</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">產品／型號</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">陪同人員</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">備註</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3358,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NCR-2026-001-jiurun</t>
+          <t xml:space="preserve">NCR-2026-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4482,17 +4382,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">依據引用</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">證書範圍</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">證書編號</t>
+          <t xml:space="preserve">適用依據引用</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4394,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2015/Amd 1:2024</t>
+          <t xml:space="preserve">2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4527,6 +4417,26 @@
       <c r="C5" t="inlineStr">
         <is>
           <t xml:space="preserve">待確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">共用管理系統認證證書</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">證書範圍</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">證書編號／引用</t>
         </is>
       </c>
     </row>
@@ -4563,7 +4473,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">公司或機構</t>
+          <t xml:space="preserve">所屬單位</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -4610,7 +4520,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">九潤精密</t>
+          <t xml:space="preserve">公司內部</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -4642,7 +4552,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">九潤精密</t>
+          <t xml:space="preserve">公司內部</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -4674,7 +4584,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">九潤精密</t>
+          <t xml:space="preserve">公司內部</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -4706,7 +4616,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">正隆興精密</t>
+          <t xml:space="preserve">公司內部</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">

</xml_diff>

<commit_message>
chore(release): refresh xlsx smoke artifact
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/release/xlsx-smoke.xlsx
+++ b/artifacts/release/xlsx-smoke.xlsx
@@ -3306,50 +3306,55 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t xml:space="preserve">公司</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t xml:space="preserve">流程</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t xml:space="preserve">要求快照</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t xml:space="preserve">證據快照</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t xml:space="preserve">發現快照</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t xml:space="preserve">日期</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t xml:space="preserve">狀態</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t xml:space="preserve">矯正措施</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t xml:space="preserve">效果確認</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t xml:space="preserve">確認人</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t xml:space="preserve">確認日</t>
         </is>
@@ -3371,22 +3376,22 @@
           <t xml:space="preserve">品保部</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t xml:space="preserve">製程/最終檢驗</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t xml:space="preserve">不合格品隔離區標示不完整</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-03-15</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t xml:space="preserve">矯正中</t>
         </is>

</xml_diff>

<commit_message>
feat(storage): v15 single workspace and formal record location gate
Complete browser-side v15 migration, settings dialog for archive path, and UI alignment fixes; remove legacy migration gate UI.
</commit_message>
<xml_diff>
--- a/artifacts/release/xlsx-smoke.xlsx
+++ b/artifacts/release/xlsx-smoke.xlsx
@@ -6,13 +6,15 @@
     <sheet name="02_QP-28_2026-02-15" sheetId="2" r:id="rId2"/>
     <sheet name="02_QP-16_2026-06-15" sheetId="3" r:id="rId3"/>
     <sheet name="02_QP-20_2026-04-15" sheetId="4" r:id="rId4"/>
-    <sheet name="QR-28-03" sheetId="5" r:id="rId5"/>
-    <sheet name="QR-02-01" sheetId="6" r:id="rId6"/>
-    <sheet name="適用標準" sheetId="7" r:id="rId7"/>
-    <sheet name="人員合格名單" sheetId="8" r:id="rId8"/>
-    <sheet name="觀察事項" sheetId="9" r:id="rId9"/>
-    <sheet name="建議追蹤" sheetId="10" r:id="rId10"/>
-    <sheet name="稽核前準備" sheetId="11" r:id="rId11"/>
+    <sheet name="02_QP-05_2026-04-15" sheetId="5" r:id="rId5"/>
+    <sheet name="02_QP-21_2026-05-15" sheetId="6" r:id="rId6"/>
+    <sheet name="QR-28-03" sheetId="7" r:id="rId7"/>
+    <sheet name="QR-02-01" sheetId="8" r:id="rId8"/>
+    <sheet name="適用標準" sheetId="9" r:id="rId9"/>
+    <sheet name="人員合格名單" sheetId="10" r:id="rId10"/>
+    <sheet name="觀察事項" sheetId="11" r:id="rId11"/>
+    <sheet name="建議追蹤" sheetId="12" r:id="rId12"/>
+    <sheet name="稽核前準備" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -1910,7 +1912,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">第三方稽核建議事項一覽表</t>
+          <t xml:space="preserve">2026 年人員合格名單</t>
         </is>
       </c>
     </row>
@@ -1918,92 +1920,175 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">年度</t>
+          <t xml:space="preserve">姓名</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">程序</t>
+          <t xml:space="preserve">編號</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">問題描述</t>
+          <t xml:space="preserve">類型</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">進度</t>
+          <t xml:space="preserve">所屬單位</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">負責單位</t>
+          <t xml:space="preserve">責任單位</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t xml:space="preserve">角色</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t xml:space="preserve">狀態</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">適用範圍</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">有效日期</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <v>2025</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">王大明</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-18</t>
+          <t xml:space="preserve">JR-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">部分量測設備校正標籤資訊不完整</t>
+          <t xml:space="preserve">內部</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">已通知各單位補貼，待複查</t>
+          <t xml:space="preserve">公司內部</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">待追蹤</t>
+          <t xml:space="preserve">dept-admin</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">待確認</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <v>2025</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">王稽核</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-09</t>
+          <t xml:space="preserve">JR-QA-01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">合約審查紀錄缺少客戶特殊要求欄位</t>
+          <t xml:space="preserve">內部</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">表單已修訂，舊案補登中</t>
+          <t xml:space="preserve">公司內部</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">業務部</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">待追蹤</t>
+          <t xml:space="preserve">dept-qa</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">待確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">李稽核</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JR-PR-01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">內部</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公司內部</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dept-prod</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">待確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">陳稽核</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZLX-001</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">內部</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公司內部</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dept-admin</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">待確認</t>
         </is>
       </c>
     </row>
@@ -2017,6 +2102,355 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t xml:space="preserve">觀察事項紀錄台帳</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">年度</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">來源</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">來源事件／報告</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">發生日</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">部門</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">觀察事項</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">說明</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">責任人</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">到期日</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">狀態</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">結案日</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">結案證據</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">追蹤時間軸</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obs-2025-1-jiurun</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>2025</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">內部稽核</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-01</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">管理部</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">文件回收舊版時，部分部門未簽收確認</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">建議強化文件發放回收簽收紀錄</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">open</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obs-2025-2-jiurun</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>2025</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">內部稽核</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-22</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生產製造部</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">工單與現場實際用料偶有不一致</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">建議每班首件核對工單物料</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">open</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obs-2025-1-zlx</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>2025</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">內部稽核</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-12</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">供應商材質證明更新不及時</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已列管追蹤，待供應商回覆</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">open</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">第三方稽核建議事項一覽表</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">年度</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">程序</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">問題描述</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">進度</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">負責單位</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">狀態</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>2025</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-18</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">部分量測設備校正標籤資訊不完整</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已通知各單位補貼，待複查</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">待追蹤</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>2025</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-09</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合約審查紀錄缺少客戶特殊要求欄位</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">表單已修訂，舊案補登中</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">業務部</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">待追蹤</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-07</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">教育訓練矩陣未含新進人員</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HR 補登中</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">管理部</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">待追蹤</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t xml:space="preserve">外部稽核前準備事項（管理代表及相關部門確認）</t>
         </is>
       </c>
@@ -2068,6 +2502,11 @@
       <c r="C5" t="inlineStr">
         <is>
           <t xml:space="preserve">品保/管理代表</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2850,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">九潤精密 · 內部稽核查檢表 QR-28-02</t>
+          <t xml:space="preserve">內部稽核工作區 · 內部稽核查檢表 QR-28-02</t>
         </is>
       </c>
     </row>
@@ -2700,7 +3139,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">九潤精密 · 內部稽核查檢表 QR-28-02</t>
+          <t xml:space="preserve">內部稽核工作區 · 內部稽核查檢表 QR-28-02</t>
         </is>
       </c>
     </row>
@@ -2999,7 +3438,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">九潤精密 · 內部稽核查檢表 QR-28-02</t>
+          <t xml:space="preserve">內部稽核工作區 · 內部稽核查檢表 QR-28-02</t>
         </is>
       </c>
     </row>
@@ -3278,122 +3717,347 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">九潤精密 · 2026 不符合事項清單 QR-28-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t xml:space="preserve">內部稽核工作區 · 內部稽核查檢表 QR-28-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-05 · 量測儀器及設備管理程序 · 系統稽核</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">NCR#</t>
+          <t xml:space="preserve">事件 ID</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">來源事件</t>
+          <t xml:space="preserve">audit-QP-05-dept-qa</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP</t>
+          <t xml:space="preserve">年度／狀態</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">部門</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公司</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">流程</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">要求快照</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">證據快照</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">發現快照</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">日期</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">狀態</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">矯正措施</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">效果確認</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">確認人</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">確認日</t>
+          <t xml:space="preserve">2026／執行中</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NCR-2026-001</t>
+          <t xml:space="preserve">適用標準快照</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-16</t>
+          <t xml:space="preserve">程序代碼／版本快照</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t xml:space="preserve">待確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">正式紀錄保存位置快照</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">快照狀態</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">稽核開始時已固定</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">團隊快照時間</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">正式回報編號</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">被稽核部門</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t xml:space="preserve">品保部</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">製程/最終檢驗</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">不合格品隔離區標示不完整</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-15</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">矯正中</t>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">稽核流程 (QP)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-05 量測儀器及設備管理程序</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">對應文件</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-05</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通知日期</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">實施日期</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-15</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">被稽核部門主管</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部經理</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">稽核人員</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">王稽核</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">團隊角色</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">姓名</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">所屬</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">資格依據</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">資格範圍</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">任命依據</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">項目</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">稽核內容</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">判定</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">內容說明</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">儀校管制</t>
+        </is>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部有無判定檢驗儀器並列入儀校管制及登錄『QR-05-01 儀器校驗一覽表』。</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">符合</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">儀器編號</t>
+        </is>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">驗收合格後,是否均應賦予唯一的儀器編號</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">儀校計畫</t>
+        </is>
+      </c>
+      <c r="B18">
+        <v>3</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是否依『QR-05-01 儀器校驗一覽表』之校驗週期要求執行校驗。 至少應包含儀器名稱、儀器識別編號、位置、使用單位、保管人、校驗頻率、校正方法、校正日期、校正結果及校正有效日期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">校驗紀錄</t>
+        </is>
+      </c>
+      <c r="B19">
+        <v>4</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">各項量儀校驗操作說明執行校驗。並將校正數據，記錄於『QR-05-03量具校驗報告』中，亦須同步更新『QR-05-01 儀器校驗一覽表』。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">三次元量測</t>
+        </is>
+      </c>
+      <c r="B20">
+        <v>5</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">每班上線是否有執行檢查在作業前,填寫『QR-05-04 三次元&amp;高度規校正紀錄表』;無檢驗需求則無須填寫紀錄表。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">校驗標籤</t>
+        </is>
+      </c>
+      <c r="B21">
+        <v>6</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">校驗後之量測儀器應貼上標籤: 檢驗合格證 /免校驗證/降級使用證/暫停使用證</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">客供儀器</t>
+        </is>
+      </c>
+      <c r="B22">
+        <v>7</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">有無客戶提供儀器設備,雖然由客戶負責校驗;而業務單位是否有填寫『QR-05-05 治工具儀器及設備申請單』</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">人員校驗資格</t>
+        </is>
+      </c>
+      <c r="B23">
+        <v>8</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">執行校驗之工作人員，有無依『QP-06 教育訓練管理程序』5.3.2 之規定,有第三方合格證書。</t>
         </is>
       </c>
     </row>
@@ -3407,173 +4071,90 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">方案風險與優先順序 QR-02-01</t>
+          <t xml:space="preserve">內部稽核工作區 · 內部稽核查檢表 QR-28-02</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">對照：NCR 0/1/2/3/≥4件→1–5；客訴／變更 無／中／高→1/3/5；距上次 ＜6/6–11/12–17/18–23/≥24月→1–5；固有 低／中／高→1/3/5；空白暫估3</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t xml:space="preserve">QP-21 · 製程與檢驗管理程序 · 系統稽核</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">事件 ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">audit-QP-21-dept-prod</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">年度／狀態</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026／執行中</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">部門</t>
+          <t xml:space="preserve">適用標準快照</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">固有風險</t>
+          <t xml:space="preserve">程序代碼／版本快照</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">上次內稽NCR</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">上次第三方NCR</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">未結NCR</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">客戶抱怨</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">重大變更</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">距上次稽核</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">優先分數</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">等級</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">暫定</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">證據</t>
+          <t xml:space="preserve">待確認</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-03</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C5">
-        <v>3</v>
-      </c>
-      <c r="J5">
-        <v>60</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
+          <t xml:space="preserve">正式紀錄保存位置快照</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">快照狀態</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">稽核開始時已固定</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-05</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C6">
-        <v>3</v>
-      </c>
-      <c r="J6">
-        <v>60</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-16</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C7">
-        <v>3</v>
-      </c>
-      <c r="J7">
-        <v>60</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">團隊快照時間</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">正式回報編號</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-04</t>
+          <t xml:space="preserve">被稽核部門</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3581,776 +4162,216 @@
           <t xml:space="preserve">生產製造部</t>
         </is>
       </c>
-      <c r="C8">
-        <v>5</v>
-      </c>
-      <c r="J8">
-        <v>66</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">稽核流程 (QP)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-21 製程與檢驗管理程序</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-26</t>
+          <t xml:space="preserve">對應文件</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">生產製造部</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>5</v>
-      </c>
-      <c r="J9">
-        <v>66</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
+          <t xml:space="preserve">QP-21</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通知日期</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-01</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">QR-28-04</t>
+          <t xml:space="preserve">實施日期</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">生產製造部</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>5</v>
-      </c>
-      <c r="J10">
-        <v>66</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
+          <t xml:space="preserve">2026-05-15</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">被稽核部門主管</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生產部經理</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-16</t>
+          <t xml:space="preserve">稽核人員</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">業務部</t>
-        </is>
-      </c>
-      <c r="C11">
-        <v>3</v>
-      </c>
-      <c r="J11">
-        <v>60</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-17</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">管理部</t>
-        </is>
-      </c>
-      <c r="C12">
-        <v>3</v>
-      </c>
-      <c r="J12">
-        <v>60</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">陳稽核</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-18</t>
+          <t xml:space="preserve">團隊角色</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">管理部</t>
-        </is>
-      </c>
-      <c r="C13">
-        <v>3</v>
-      </c>
-      <c r="J13">
-        <v>60</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-01</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C14">
-        <v>3</v>
-      </c>
-      <c r="J14">
-        <v>60</v>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">姓名</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">所屬</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">資格依據</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">資格範圍</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">任命依據</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-02</t>
+          <t xml:space="preserve">項目</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C15">
-        <v>3</v>
-      </c>
-      <c r="J15">
-        <v>60</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">稽核內容</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">判定</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">內容說明</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-08</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C16">
-        <v>3</v>
-      </c>
-      <c r="J16">
-        <v>60</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
+          <t xml:space="preserve">抽驗標準</t>
+        </is>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">根據5.6.1 產品類別對應檢驗紀錄表,檢驗紀錄表的抽樣數有無依『5.6 抽樣計畫』作業</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">觀察</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">首件檢查紀錄偶缺簽名</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-09</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C17">
-        <v>3</v>
-      </c>
-      <c r="J17">
-        <v>60</v>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
+          <t xml:space="preserve">紀錄表資料是否齊全</t>
+        </is>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">該站別完工後,需將每批加工數量、不良情況是否紀錄於『QR-11-05生產流程單』或『QR-11-04 生產途程明細表』。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-12</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C18">
+          <t xml:space="preserve">生產日報表</t>
+        </is>
+      </c>
+      <c r="B18">
         <v>3</v>
       </c>
-      <c r="J18">
-        <v>60</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生產製程單位負責將每班別生產完成之產品數量統計並紀錄於『QR-20-02 生產日報表』並回報給生管人員。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-19</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C19">
-        <v>3</v>
-      </c>
-      <c r="J19">
-        <v>60</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
+          <t xml:space="preserve">不良品處置</t>
+        </is>
+      </c>
+      <c r="B19">
+        <v>4</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">製造中產生之不合格產品應立即標示及反應，依『QP-26不合格品管理程序』之相關流程處置。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-22</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C20">
-        <v>3</v>
-      </c>
-      <c r="J20">
-        <v>60</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-25</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C21">
-        <v>3</v>
-      </c>
-      <c r="J21">
-        <v>60</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-27</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C22">
-        <v>3</v>
-      </c>
-      <c r="J22">
-        <v>60</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-28</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C23">
-        <v>3</v>
-      </c>
-      <c r="J23">
-        <v>60</v>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QR-28-05</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C24">
-        <v>3</v>
-      </c>
-      <c r="J24">
-        <v>60</v>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-21</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">生產製造部</t>
-        </is>
-      </c>
-      <c r="C25">
+          <t xml:space="preserve">異常處理</t>
+        </is>
+      </c>
+      <c r="B20">
         <v>5</v>
       </c>
-      <c r="J25">
-        <v>66</v>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-10</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">開發工程部</t>
-        </is>
-      </c>
-      <c r="C26">
-        <v>3</v>
-      </c>
-      <c r="J26">
-        <v>60</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-11</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">開發工程部</t>
-        </is>
-      </c>
-      <c r="C27">
-        <v>3</v>
-      </c>
-      <c r="J27">
-        <v>60</v>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-13</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">開發工程部</t>
-        </is>
-      </c>
-      <c r="C28">
-        <v>3</v>
-      </c>
-      <c r="J28">
-        <v>60</v>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-14</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">開發工程部</t>
-        </is>
-      </c>
-      <c r="C29">
-        <v>3</v>
-      </c>
-      <c r="J29">
-        <v>60</v>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-15</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">開發工程部</t>
-        </is>
-      </c>
-      <c r="C30">
-        <v>3</v>
-      </c>
-      <c r="J30">
-        <v>60</v>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-23</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">業務部</t>
-        </is>
-      </c>
-      <c r="C31">
-        <v>3</v>
-      </c>
-      <c r="J31">
-        <v>60</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-06</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">管理部</t>
-        </is>
-      </c>
-      <c r="C32">
-        <v>3</v>
-      </c>
-      <c r="J32">
-        <v>60</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-07</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">管理部</t>
-        </is>
-      </c>
-      <c r="C33">
-        <v>3</v>
-      </c>
-      <c r="J33">
-        <v>60</v>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-20</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">管理部</t>
-        </is>
-      </c>
-      <c r="C34">
-        <v>3</v>
-      </c>
-      <c r="J34">
-        <v>60</v>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-24</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">管理部</t>
-        </is>
-      </c>
-      <c r="C35">
-        <v>3</v>
-      </c>
-      <c r="J35">
-        <v>60</v>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">是</t>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">檢驗中發現問題時,是否將其記錄於『QR-21-04 異常問題紀錄表』。  問題解決後,是否將其記錄於『QR-21-04 異常問題紀錄表』。</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4385,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">九潤精密 · 適用標準與證書</t>
+          <t xml:space="preserve">內部稽核工作區 · 2026 不符合事項清單 QR-28-03</t>
         </is>
       </c>
     </row>
@@ -4372,76 +4393,114 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">標準</t>
+          <t xml:space="preserve">NCR#</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">版本</t>
+          <t xml:space="preserve">來源事件</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">適用性</t>
+          <t xml:space="preserve">QP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">適用依據引用</t>
+          <t xml:space="preserve">部門</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公司</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">流程</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">要求快照</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">證據快照</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">發現快照</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">日期</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">狀態</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">矯正措施</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">效果確認</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">確認人</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">確認日</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISO 9001</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026</t>
+          <t xml:space="preserve">NCR-2026-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">待確認</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AS9100</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2016 (Rev D)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">待確認</t>
-        </is>
-      </c>
-    </row>
-    <row r="6"/>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">共用管理系統認證證書</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">證書範圍</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">證書編號／引用</t>
+          <t xml:space="preserve">QP-16</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">製程/最終檢驗</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">不合格品隔離區標示不完整</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-15</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">矯正中</t>
         </is>
       </c>
     </row>
@@ -4455,183 +4514,950 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026 年人員合格名單</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">姓名</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">編號</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">類型</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">所屬單位</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">責任單位</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">角色</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">狀態</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">適用範圍</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">有效日期</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">方案風險與優先順序 QR-02-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">對照：NCR 0/1/2/3/≥4件→1–5；客訴／變更 無／中／高→1/3/5；距上次 ＜6/6–11/12–17/18–23/≥24月→1–5；固有 低／中／高→1/3/5；空白暫估3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">王大明</t>
+          <t xml:space="preserve">QP</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">JR-001</t>
+          <t xml:space="preserve">部門</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">內部</t>
+          <t xml:space="preserve">固有風險</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">公司內部</t>
+          <t xml:space="preserve">上次內稽NCR</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">dept-admin</t>
+          <t xml:space="preserve">上次第三方NCR</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未結NCR</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">待確認</t>
+          <t xml:space="preserve">客戶抱怨</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">重大變更</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">距上次稽核</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">優先分數</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">等級</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">暫定</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">證據</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">王稽核</t>
+          <t xml:space="preserve">QP-03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">JR-QA-01</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">內部</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公司內部</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dept-qa</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">待確認</t>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>60</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">李稽核</t>
+          <t xml:space="preserve">QP-05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">JR-PR-01</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">內部</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公司內部</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dept-prod</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">待確認</t>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="J6">
+        <v>60</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">陳稽核</t>
+          <t xml:space="preserve">QP-16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZLX-001</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">內部</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公司內部</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dept-admin</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">待確認</t>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="J7">
+        <v>60</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-04</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生產製造部</t>
+        </is>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="J8">
+        <v>66</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-26</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生產製造部</t>
+        </is>
+      </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
+      <c r="J9">
+        <v>66</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QR-28-04</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生產製造部</t>
+        </is>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="J10">
+        <v>66</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-16</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">業務部</t>
+        </is>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="J11">
+        <v>60</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-17</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">管理部</t>
+        </is>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="J12">
+        <v>60</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-18</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">管理部</t>
+        </is>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="J13">
+        <v>60</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-01</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="J14">
+        <v>60</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-02</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
+      <c r="J15">
+        <v>60</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-08</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="J16">
+        <v>60</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>60</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-12</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C18">
+        <v>3</v>
+      </c>
+      <c r="J18">
+        <v>60</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-19</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C19">
+        <v>3</v>
+      </c>
+      <c r="J19">
+        <v>60</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-22</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C20">
+        <v>3</v>
+      </c>
+      <c r="J20">
+        <v>60</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C21">
+        <v>3</v>
+      </c>
+      <c r="J21">
+        <v>60</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-27</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="J22">
+        <v>60</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C23">
+        <v>3</v>
+      </c>
+      <c r="J23">
+        <v>60</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QR-28-05</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品保部</t>
+        </is>
+      </c>
+      <c r="C24">
+        <v>3</v>
+      </c>
+      <c r="J24">
+        <v>60</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-21</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生產製造部</t>
+        </is>
+      </c>
+      <c r="C25">
+        <v>5</v>
+      </c>
+      <c r="J25">
+        <v>66</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-10</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">開發工程部</t>
+        </is>
+      </c>
+      <c r="C26">
+        <v>3</v>
+      </c>
+      <c r="J26">
+        <v>60</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-11</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">開發工程部</t>
+        </is>
+      </c>
+      <c r="C27">
+        <v>3</v>
+      </c>
+      <c r="J27">
+        <v>60</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-13</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">開發工程部</t>
+        </is>
+      </c>
+      <c r="C28">
+        <v>3</v>
+      </c>
+      <c r="J28">
+        <v>60</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-14</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">開發工程部</t>
+        </is>
+      </c>
+      <c r="C29">
+        <v>3</v>
+      </c>
+      <c r="J29">
+        <v>60</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-15</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">開發工程部</t>
+        </is>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="J30">
+        <v>60</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-23</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">業務部</t>
+        </is>
+      </c>
+      <c r="C31">
+        <v>3</v>
+      </c>
+      <c r="J31">
+        <v>60</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-06</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">管理部</t>
+        </is>
+      </c>
+      <c r="C32">
+        <v>3</v>
+      </c>
+      <c r="J32">
+        <v>60</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-07</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">管理部</t>
+        </is>
+      </c>
+      <c r="C33">
+        <v>3</v>
+      </c>
+      <c r="J33">
+        <v>60</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-20</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">管理部</t>
+        </is>
+      </c>
+      <c r="C34">
+        <v>3</v>
+      </c>
+      <c r="J34">
+        <v>60</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-24</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">管理部</t>
+        </is>
+      </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
+      <c r="J35">
+        <v>60</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
         </is>
       </c>
     </row>
@@ -4645,7 +5471,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">觀察事項紀錄台帳</t>
+          <t xml:space="preserve">內部稽核工作區 · 適用標準與證書</t>
         </is>
       </c>
     </row>
@@ -4653,157 +5479,76 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID</t>
+          <t xml:space="preserve">標準</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">年度</t>
+          <t xml:space="preserve">版本</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">來源</t>
+          <t xml:space="preserve">適用性</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">來源事件／報告</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">發生日</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">部門</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">觀察事項</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">說明</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">責任人</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">到期日</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">狀態</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">結案日</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">結案證據</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">追蹤時間軸</t>
+          <t xml:space="preserve">適用依據引用</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">obs-2025-1-jiurun</t>
-        </is>
-      </c>
-      <c r="B4">
-        <v>2025</v>
+          <t xml:space="preserve">ISO 9001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">內部稽核</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-01</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">管理部</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">文件回收舊版時，部分部門未簽收確認</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">建議強化文件發放回收簽收紀錄</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">open</t>
+          <t xml:space="preserve">待確認</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">obs-2025-2-jiurun</t>
-        </is>
-      </c>
-      <c r="B5">
-        <v>2025</v>
+          <t xml:space="preserve">AS9100</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2016 (Rev D)</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">內部稽核</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP-22</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">生產製造部</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">工單與現場實際用料偶有不一致</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">建議每班首件核對工單物料</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">open</t>
+          <t xml:space="preserve">待確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">共用管理系統認證證書</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">證書範圍</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">證書編號／引用</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: prepare production release and fix lint
</commit_message>
<xml_diff>
--- a/artifacts/release/xlsx-smoke.xlsx
+++ b/artifacts/release/xlsx-smoke.xlsx
@@ -1990,9 +1990,24 @@
           <t xml:space="preserve">dept-admin</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合格內部稽核員</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">待確認</t>
+          <t xml:space="preserve">有效</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ISO 9001:2015、AS9100:2016 (Rev D)／QP-28／dept-admin</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-01～正式依據未訂期限</t>
         </is>
       </c>
     </row>
@@ -2022,9 +2037,24 @@
           <t xml:space="preserve">dept-qa</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合格內部稽核員</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">待確認</t>
+          <t xml:space="preserve">有效</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ISO 9001:2015、AS9100:2016 (Rev D)／QP-28／dept-qa</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-01～正式依據未訂期限</t>
         </is>
       </c>
     </row>
@@ -2054,9 +2084,24 @@
           <t xml:space="preserve">dept-prod</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">實習稽核員</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">待確認</t>
+          <t xml:space="preserve">有效</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ISO 9001:2015、AS9100:2016 (Rev D)／QP-28／dept-qa</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-01～正式依據未訂期限</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(audit): fold external-audit prep into the checklist page as a view; single source via linkedQp, single control for item 4 and management review
</commit_message>
<xml_diff>
--- a/artifacts/release/xlsx-smoke.xlsx
+++ b/artifacts/release/xlsx-smoke.xlsx
@@ -2526,10 +2526,15 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t xml:space="preserve">關聯查檢</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t xml:space="preserve">完成</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t xml:space="preserve">備註</t>
         </is>
@@ -2551,6 +2556,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t xml:space="preserve">QP-08 品保部</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t xml:space="preserve">是</t>
         </is>
       </c>
@@ -2569,6 +2579,11 @@
           <t xml:space="preserve">品保彙整／各部門繳交</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-28 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -2584,6 +2599,11 @@
           <t xml:space="preserve">稽核員</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-28 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -2599,6 +2619,11 @@
           <t xml:space="preserve">稽核員</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-28 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -2614,6 +2639,11 @@
           <t xml:space="preserve">品保彙整／管理代表／各責任部門</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-03 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -2629,6 +2659,11 @@
           <t xml:space="preserve">管理代表／品保</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-03 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -2644,6 +2679,11 @@
           <t xml:space="preserve">責任單位／品保</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-02 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -2659,6 +2699,11 @@
           <t xml:space="preserve">品保/各主管</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-03 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -2674,6 +2719,11 @@
           <t xml:space="preserve">管理代表</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-01 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -2689,6 +2739,11 @@
           <t xml:space="preserve">品保(文管)</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-08 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -2704,6 +2759,11 @@
           <t xml:space="preserve">各部門</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-09 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -2719,6 +2779,11 @@
           <t xml:space="preserve">生產製造部</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-04 生產製造部</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -2734,6 +2799,11 @@
           <t xml:space="preserve">全廠區</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-26 生產製造部</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -2749,6 +2819,11 @@
           <t xml:space="preserve">各部門/人資</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-06 管理部</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -2764,6 +2839,11 @@
           <t xml:space="preserve">開發工程</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-11 開發工程部、QP-14 開發工程部</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -2779,6 +2859,11 @@
           <t xml:space="preserve">業務部</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-16 業務部、QP-16 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -2794,6 +2879,11 @@
           <t xml:space="preserve">外包/採購/開發工程</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-17 管理部、QP-18 管理部</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -2809,6 +2899,11 @@
           <t xml:space="preserve">倉儲</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-24 管理部</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -2824,6 +2919,11 @@
           <t xml:space="preserve">生產製造</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QR-28-04 生產製造部</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -2839,6 +2939,11 @@
           <t xml:space="preserve">生產製造</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-04 生產製造部</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -2854,6 +2959,11 @@
           <t xml:space="preserve">品保</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-05 品保部</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -2869,6 +2979,11 @@
           <t xml:space="preserve">業務/開發工程</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-10 開發工程部</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -2882,6 +2997,11 @@
       <c r="C27" t="inlineStr">
         <is>
           <t xml:space="preserve">品保</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QP-19 品保部、QP-25 品保部</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP: epitaxy pre-switch from work/risk-assessment-p0
</commit_message>
<xml_diff>
--- a/artifacts/release/xlsx-smoke.xlsx
+++ b/artifacts/release/xlsx-smoke.xlsx
@@ -4686,110 +4686,109 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">對照：NCR 0/1/2/3/≥4件→1–5；客訴／變更 無／中／高→1/3/5；距上次 ＜6/6–11/12–17/18–23/≥24月→1–5；固有 低／中／高→1/3/5；空白暫估3</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QP</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">部門</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">固有風險</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">上次內稽NCR</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">上次第三方NCR</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">未結NCR</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">客戶抱怨</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">重大變更</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">距上次稽核</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">優先分數</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">等級</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">暫定</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">證據</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">對照：NCR／客訴／重大變更 0/1/2/3/≥4件→1–5；距上次 ＜6/6–11/12–17/18–23/≥24月→1–5；固有 低／中／高→1/3/5（預設取程序種子）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">空白＝資料不足（不給等級、不參與編排）；未取得須註明理由並以 3 計分；固有高者等級至少為中（公司自訂規則，非標準要求）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-03</t>
+          <t xml:space="preserve">QP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">品保部</t>
-        </is>
-      </c>
-      <c r="C5">
-        <v>3</v>
-      </c>
-      <c r="J5">
-        <v>60</v>
+          <t xml:space="preserve">部門</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">固有風險</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上次內稽NCR</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上次第三方NCR</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未結NCR</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">客戶抱怨件數</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">重大變更件數</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">距上次稽核</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">優先分數</t>
+        </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">等級</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t xml:space="preserve">是</t>
+          <t xml:space="preserve">暫定</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">證據</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">狀態</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">評估年度</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未取得因子</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">固有地板</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-05</t>
+          <t xml:space="preserve">QP-03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4805,19 +4804,24 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-16</t>
+          <t xml:space="preserve">QP-05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4833,47 +4837,57 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-04</t>
+          <t xml:space="preserve">QP-16</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">生產製造部</t>
+          <t xml:space="preserve">品保部</t>
         </is>
       </c>
       <c r="C8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J8">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-26</t>
+          <t xml:space="preserve">QP-04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4882,26 +4896,31 @@
         </is>
       </c>
       <c r="C9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J9">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">QR-28-04</t>
+          <t xml:space="preserve">QP-26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4910,31 +4929,36 @@
         </is>
       </c>
       <c r="C10">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J10">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-16</t>
+          <t xml:space="preserve">QR-28-04</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">業務部</t>
+          <t xml:space="preserve">生產製造部</t>
         </is>
       </c>
       <c r="C11">
@@ -4945,24 +4969,29 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-17</t>
+          <t xml:space="preserve">QP-16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">管理部</t>
+          <t xml:space="preserve">業務部</t>
         </is>
       </c>
       <c r="C12">
@@ -4973,19 +5002,24 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-18</t>
+          <t xml:space="preserve">QP-17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -5001,24 +5035,29 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-01</t>
+          <t xml:space="preserve">QP-18</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">品保部</t>
+          <t xml:space="preserve">管理部</t>
         </is>
       </c>
       <c r="C14">
@@ -5029,19 +5068,24 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-02</t>
+          <t xml:space="preserve">QP-01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -5050,26 +5094,31 @@
         </is>
       </c>
       <c r="C15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J15">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-08</t>
+          <t xml:space="preserve">QP-02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5078,26 +5127,31 @@
         </is>
       </c>
       <c r="C16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J16">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-09</t>
+          <t xml:space="preserve">QP-08</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -5106,26 +5160,31 @@
         </is>
       </c>
       <c r="C17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J17">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-12</t>
+          <t xml:space="preserve">QP-09</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -5134,26 +5193,31 @@
         </is>
       </c>
       <c r="C18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-19</t>
+          <t xml:space="preserve">QP-12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -5162,26 +5226,31 @@
         </is>
       </c>
       <c r="C19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J19">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-22</t>
+          <t xml:space="preserve">QP-19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5190,26 +5259,31 @@
         </is>
       </c>
       <c r="C20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J20">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-25</t>
+          <t xml:space="preserve">QP-22</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -5218,26 +5292,31 @@
         </is>
       </c>
       <c r="C21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J21">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-27</t>
+          <t xml:space="preserve">QP-25</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5246,26 +5325,31 @@
         </is>
       </c>
       <c r="C22">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J22">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-28</t>
+          <t xml:space="preserve">QP-27</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5274,26 +5358,31 @@
         </is>
       </c>
       <c r="C23">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J23">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">QR-28-05</t>
+          <t xml:space="preserve">QP-28</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5302,82 +5391,97 @@
         </is>
       </c>
       <c r="C24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J24">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-21</t>
+          <t xml:space="preserve">QR-28-05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">生產製造部</t>
+          <t xml:space="preserve">品保部</t>
         </is>
       </c>
       <c r="C25">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J25">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-10</t>
+          <t xml:space="preserve">QP-21</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">開發工程部</t>
+          <t xml:space="preserve">生產製造部</t>
         </is>
       </c>
       <c r="C26">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J26">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-11</t>
+          <t xml:space="preserve">QP-10</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5386,26 +5490,31 @@
         </is>
       </c>
       <c r="C27">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J27">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-13</t>
+          <t xml:space="preserve">QP-11</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5414,26 +5523,31 @@
         </is>
       </c>
       <c r="C28">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J28">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-14</t>
+          <t xml:space="preserve">QP-13</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5442,26 +5556,31 @@
         </is>
       </c>
       <c r="C29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J29">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-15</t>
+          <t xml:space="preserve">QP-14</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5470,82 +5589,97 @@
         </is>
       </c>
       <c r="C30">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J30">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-23</t>
+          <t xml:space="preserve">QP-15</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">業務部</t>
+          <t xml:space="preserve">開發工程部</t>
         </is>
       </c>
       <c r="C31">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J31">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-06</t>
+          <t xml:space="preserve">QP-23</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">管理部</t>
+          <t xml:space="preserve">業務部</t>
         </is>
       </c>
       <c r="C32">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J32">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-07</t>
+          <t xml:space="preserve">QP-06</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5554,26 +5688,31 @@
         </is>
       </c>
       <c r="C33">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J33">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">QP-20</t>
+          <t xml:space="preserve">QP-07</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5582,47 +5721,90 @@
         </is>
       </c>
       <c r="C34">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J34">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">資料不足</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t xml:space="preserve">QP-20</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">管理部</t>
+        </is>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="J35">
+        <v>54</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">資料不足</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t xml:space="preserve">QP-24</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t xml:space="preserve">管理部</t>
         </is>
       </c>
-      <c r="C35">
-        <v>3</v>
-      </c>
-      <c r="J35">
-        <v>60</v>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="J36">
+        <v>54</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">資料不足</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未評估</t>
         </is>
       </c>
     </row>

</xml_diff>